<commit_message>
fix: correct Sprint Plan status cell formatting to match existing styles
Status cells for rows S2-08, S3-05, S4-04, S7-07 now use the same
Arial 10pt + green fill as other "Complete" cells. S6-05 "Partial"
matches the existing amber style.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Operations/Waypoint-GTM-IT-Project-Plan-v1.xlsx
+++ b/Operations/Waypoint-GTM-IT-Project-Plan-v1.xlsx
@@ -1614,7 +1614,7 @@
           <t>S2 / W2</t>
         </is>
       </c>
-      <c r="G24" s="39" t="inlineStr">
+      <c r="G24" s="35" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -1944,7 +1944,7 @@
           <t>S3 / W4</t>
         </is>
       </c>
-      <c r="G32" s="39" t="inlineStr">
+      <c r="G32" s="35" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2274,7 +2274,7 @@
           <t>S4 / W6</t>
         </is>
       </c>
-      <c r="G40" s="40" t="inlineStr">
+      <c r="G40" s="35" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -2979,7 +2979,7 @@
           <t>S6 / W10</t>
         </is>
       </c>
-      <c r="G57" s="42" t="inlineStr">
+      <c r="G57" s="39" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -3444,7 +3444,7 @@
           <t>S7 / W11</t>
         </is>
       </c>
-      <c r="G68" s="42" t="inlineStr">
+      <c r="G68" s="35" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>

</xml_diff>